<commit_message>
Finish purchse screen work
</commit_message>
<xml_diff>
--- a/Management Portal/Tables name and column.xlsx
+++ b/Management Portal/Tables name and column.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New project\Management Portal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1DD3A8F-71CB-457F-A84E-2B64E6C67283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF24A72-65D3-4D39-98D3-B5FCB0B230C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$N$45</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="64">
   <si>
     <t>tbl_Category</t>
   </si>
@@ -213,7 +213,13 @@
     <t>Priority</t>
   </si>
   <si>
-    <t>S</t>
+    <t>W</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>line</t>
   </si>
 </sst>
 </file>
@@ -559,17 +565,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M45"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>46</v>
       </c>
@@ -585,28 +592,31 @@
       <c r="E1" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="4"/>
+      <c r="J1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="4"/>
+      <c r="M1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +627,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -628,15 +638,24 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>1.3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -644,15 +663,21 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -660,15 +685,21 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -679,7 +710,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -693,15 +724,21 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -709,7 +746,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -723,7 +760,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -731,7 +768,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -742,7 +779,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -753,7 +790,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -764,7 +801,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -775,7 +812,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -783,7 +820,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -797,7 +834,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -805,7 +842,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -813,7 +850,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -824,7 +861,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -832,7 +869,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -840,18 +877,24 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B26" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="D26">
+        <v>2.1</v>
+      </c>
+      <c r="E26" t="s">
+        <v>62</v>
+      </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -859,7 +902,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -870,7 +913,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -881,7 +924,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -892,7 +935,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>29</v>
       </c>
@@ -903,21 +946,21 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B32" t="s">
         <v>44</v>
       </c>
-      <c r="D32">
-        <v>1.3</v>
-      </c>
       <c r="E32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+      <c r="F32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -928,29 +971,35 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
-      </c>
-      <c r="C34" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E34" t="s">
+        <v>62</v>
+      </c>
+      <c r="F34">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="B35" t="s">
         <v>44</v>
       </c>
       <c r="E35" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+      <c r="F35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -958,7 +1007,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -966,15 +1015,24 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="C38" t="s">
+        <v>50</v>
+      </c>
+      <c r="E38" t="s">
+        <v>62</v>
+      </c>
+      <c r="F38">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -982,26 +1040,35 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
-      </c>
-      <c r="D40">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="C40" t="s">
+        <v>50</v>
+      </c>
+      <c r="E40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F40">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
       <c r="B41" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E41" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>40</v>
       </c>
@@ -1012,15 +1079,18 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>42</v>
       </c>
@@ -1031,7 +1101,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>59</v>
       </c>
@@ -1043,7 +1113,21 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M45" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:N45" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters blank="1">
+        <filter val="It Wiil Fill By database"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="w"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:N43">
+      <sortCondition ref="F1:F45"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>